<commit_message>
Report: From / To date dropdowns that recompute the page client-side
The HTML report now has From, To and Quick range (month) dropdowns. Choosing a
range recomputes tiles, billed time, the calendar (days outside the range dimmed),
meetings and tasks in the browser; ?from=&to= preselects a range. Per-day values are
embedded from the recalculated workbook. The CSP allows exactly one inline script,
pinned by SHA-256; fixtures check the pin, the dropdowns and the script syntax.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/examples/example.xlsx
+++ b/assets/examples/example.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timot\Documents\projects\org-comms-export-skill\tests\out\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timot\Documents\projects\org-time-tracking-skill\tests\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C22B6CE-D33B-4645-A6FA-D9188B658733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242E60EF-154E-490A-9EFD-2CA6A484E4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="990" yWindow="2835" windowWidth="22785" windowHeight="17895" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -721,7 +721,7 @@
     <t>Transaction log file size crossed threshold</t>
   </si>
   <si>
-    <t>Email times are not recorded (list view only). Teams times are America/New_York. Secrets are redacted. Source: C:\Users\timot\Documents\projects\org-comms-export-skill\tests\out\./tree</t>
+    <t>Email times are not recorded (list view only). Teams times are America/New_York. Secrets are redacted. Source: C:\Users\timot\Documents\projects\org-time-tracking-skill\tests\out\./tree</t>
   </si>
   <si>
     <t>Alert type</t>

</xml_diff>

<commit_message>
Add a client logo spot (org.logo) beside the brand mark
org.logo takes a local image file for the client's own mark. It appears next to the
brand logo in the workbook banner and at the right of the report header (on a white
tile so it stays legible in dark mode). Remote/data-URI logos, non-image files and
files over 2 MB are rejected; logos/ and client-logo.* are git- and bundle-ignored.
The example render uses a fictional Northwind wordmark.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/examples/example.xlsx
+++ b/assets/examples/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timot\Documents\projects\org-time-tracking-skill\tests\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242E60EF-154E-490A-9EFD-2CA6A484E4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62187088-5696-4567-BF0E-2EDA0BD1587D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="990" yWindow="2835" windowWidth="22785" windowHeight="17895" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -989,7 +989,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1428750" cy="704850"/>
+    <xdr:ext cx="1066800" cy="533400"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
@@ -1003,6 +1003,39 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2000250" cy="533400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>

</xml_diff>